<commit_message>
Normalize encounter rates to exactly 100% per location and method
- Normalizes the base weights of Pokemon mapped from 'Common', 'Rare', etc. so that they sum to exactly 100.00% for each location and method.
- Utilizes Largest Remainder Method (LRM) for floating point precision.
- Re-generates `Johto.xlsx` to reflect accurate percentages and grouping.

Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Johto.xlsx
+++ b/Johto.xlsx
@@ -466,7 +466,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>11.77%</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>5.88%</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>23.53%</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>15%, 30%, 5%</t>
+          <t>10.78%</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.98%</t>
         </is>
       </c>
     </row>
@@ -601,7 +601,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>11.77%</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.94%</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.94%</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>11.77%</t>
         </is>
       </c>
     </row>
@@ -709,7 +709,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>5.88%</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>5.88%</t>
         </is>
       </c>
     </row>
@@ -763,7 +763,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>5.88%</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.41%</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>30%, 5%</t>
+          <t>5.15%</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>11.03%</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.41%</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>17.65%</t>
         </is>
       </c>
     </row>
@@ -925,7 +925,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>6.62%</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>6.62%</t>
         </is>
       </c>
     </row>
@@ -979,7 +979,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.74%</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.74%</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.73%</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>4.41%</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1087,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>4.41%</t>
         </is>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.21%</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1195,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1303,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1330,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>8.82%</t>
         </is>
       </c>
     </row>
@@ -1411,7 +1411,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>8.82%</t>
         </is>
       </c>
     </row>
@@ -1438,7 +1438,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>4.41%</t>
         </is>
       </c>
     </row>
@@ -1465,7 +1465,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.41%</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.41%</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>8.11%</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>30%, 5%</t>
+          <t>4.73%</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1573,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>10.14%</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.06%</t>
         </is>
       </c>
     </row>
@@ -1627,7 +1627,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>14.19%</t>
         </is>
       </c>
     </row>
@@ -1654,7 +1654,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>6.08%</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1681,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>6.08%</t>
         </is>
       </c>
     </row>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.05%</t>
         </is>
       </c>
     </row>
@@ -1735,7 +1735,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.68%</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.68%</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.68%</t>
         </is>
       </c>
     </row>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>4.05%</t>
         </is>
       </c>
     </row>
@@ -1843,7 +1843,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>4.05%</t>
         </is>
       </c>
     </row>
@@ -1870,7 +1870,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>4.05%</t>
         </is>
       </c>
     </row>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1924,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -2032,7 +2032,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -2059,7 +2059,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2113,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>8.11%</t>
         </is>
       </c>
     </row>
@@ -2167,7 +2167,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>8.11%</t>
         </is>
       </c>
     </row>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>4.05%</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.05%</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2248,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.05%</t>
         </is>
       </c>
     </row>
@@ -2275,7 +2275,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>15%, 30%, 5%</t>
+          <t>21.05%</t>
         </is>
       </c>
     </row>
@@ -2302,7 +2302,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>6.77%</t>
         </is>
       </c>
     </row>
@@ -2329,7 +2329,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>9.02%</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>30%, 5%</t>
+          <t>9.78%</t>
         </is>
       </c>
     </row>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>15%, 5%</t>
+          <t>3.76%</t>
         </is>
       </c>
     </row>
@@ -2410,7 +2410,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.75%</t>
         </is>
       </c>
     </row>
@@ -2437,7 +2437,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.75%</t>
         </is>
       </c>
     </row>
@@ -2464,7 +2464,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>30%, 5%</t>
+          <t>9.78%</t>
         </is>
       </c>
     </row>
@@ -2491,7 +2491,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.26%</t>
         </is>
       </c>
     </row>
@@ -2518,7 +2518,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>4.51%</t>
         </is>
       </c>
     </row>
@@ -2545,7 +2545,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>40.00%</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2572,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>40.00%</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2599,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>20.00%</t>
         </is>
       </c>
     </row>
@@ -2626,7 +2626,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -2653,7 +2653,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>16.67%</t>
         </is>
       </c>
     </row>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -2707,7 +2707,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>20.00%</t>
         </is>
       </c>
     </row>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>40.00%</t>
         </is>
       </c>
     </row>
@@ -2761,7 +2761,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>40.00%</t>
         </is>
       </c>
     </row>
@@ -2788,7 +2788,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.66%</t>
         </is>
       </c>
     </row>
@@ -2815,7 +2815,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>16.67%</t>
         </is>
       </c>
     </row>
@@ -2842,7 +2842,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>16.67%</t>
         </is>
       </c>
     </row>
@@ -2869,7 +2869,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>9.02%</t>
         </is>
       </c>
     </row>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>9.02%</t>
         </is>
       </c>
     </row>
@@ -2923,7 +2923,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>4.51%</t>
         </is>
       </c>
     </row>
@@ -2950,7 +2950,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.51%</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.51%</t>
         </is>
       </c>
     </row>
@@ -3004,7 +3004,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>17.65%</t>
         </is>
       </c>
     </row>
@@ -3031,7 +3031,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>15%, 30%, 5%</t>
+          <t>8.40%</t>
         </is>
       </c>
     </row>
@@ -3058,7 +3058,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>30%, 5%</t>
+          <t>10.93%</t>
         </is>
       </c>
     </row>
@@ -3085,7 +3085,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>7.56%</t>
         </is>
       </c>
     </row>
@@ -3112,7 +3112,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>27.73%</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.52%</t>
         </is>
       </c>
     </row>
@@ -3166,7 +3166,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>15.13%</t>
         </is>
       </c>
     </row>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>10.08%</t>
         </is>
       </c>
     </row>
@@ -3220,7 +3220,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>9.76%</t>
         </is>
       </c>
     </row>
@@ -3247,7 +3247,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>9.76%</t>
         </is>
       </c>
     </row>
@@ -3274,7 +3274,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.88%</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3301,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.81%</t>
         </is>
       </c>
     </row>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.81%</t>
         </is>
       </c>
     </row>
@@ -3355,7 +3355,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.44%</t>
         </is>
       </c>
     </row>
@@ -3382,7 +3382,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.44%</t>
         </is>
       </c>
     </row>
@@ -3409,7 +3409,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>12.19%</t>
         </is>
       </c>
     </row>
@@ -3436,7 +3436,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -3490,7 +3490,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>28.57%</t>
         </is>
       </c>
     </row>
@@ -3517,7 +3517,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>28.57%</t>
         </is>
       </c>
     </row>
@@ -3544,7 +3544,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>28.57%</t>
         </is>
       </c>
     </row>
@@ -3571,7 +3571,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>14.29%</t>
         </is>
       </c>
     </row>
@@ -3598,7 +3598,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -3625,7 +3625,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -3652,7 +3652,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>16.67%</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>16.67%</t>
         </is>
       </c>
     </row>
@@ -3706,7 +3706,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -3760,7 +3760,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>14.29%</t>
         </is>
       </c>
     </row>
@@ -3787,7 +3787,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>14.29%</t>
         </is>
       </c>
     </row>
@@ -3814,7 +3814,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>14.29%</t>
         </is>
       </c>
     </row>
@@ -3841,7 +3841,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>14.29%</t>
         </is>
       </c>
     </row>
@@ -3868,7 +3868,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>14.28%</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3895,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>14.28%</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>14.28%</t>
         </is>
       </c>
     </row>
@@ -3949,7 +3949,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>14.63%</t>
         </is>
       </c>
     </row>
@@ -3976,7 +3976,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.44%</t>
         </is>
       </c>
     </row>
@@ -4003,7 +4003,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.44%</t>
         </is>
       </c>
     </row>
@@ -4030,7 +4030,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>9.76%</t>
         </is>
       </c>
     </row>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>9.76%</t>
         </is>
       </c>
     </row>
@@ -4084,7 +4084,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1.62%</t>
         </is>
       </c>
     </row>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1.62%</t>
         </is>
       </c>
     </row>
@@ -4138,7 +4138,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.44%</t>
         </is>
       </c>
     </row>
@@ -4165,7 +4165,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.44%</t>
         </is>
       </c>
     </row>
@@ -4192,7 +4192,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>9.76%</t>
         </is>
       </c>
     </row>
@@ -4219,7 +4219,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>7.69%</t>
         </is>
       </c>
     </row>
@@ -4246,7 +4246,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>7.69%</t>
         </is>
       </c>
     </row>
@@ -4273,7 +4273,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>30%, 5%</t>
+          <t>5.13%</t>
         </is>
       </c>
     </row>
@@ -4300,7 +4300,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>5.77%</t>
         </is>
       </c>
     </row>
@@ -4327,7 +4327,7 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>30%, 5%</t>
+          <t>12.18%</t>
         </is>
       </c>
     </row>
@@ -4354,7 +4354,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>3.85%</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4381,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1.28%</t>
         </is>
       </c>
     </row>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>30%, 5%</t>
+          <t>4.49%</t>
         </is>
       </c>
     </row>
@@ -4435,7 +4435,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.64%</t>
         </is>
       </c>
     </row>
@@ -4462,7 +4462,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>1.93%</t>
         </is>
       </c>
     </row>
@@ -4489,7 +4489,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>1.93%</t>
         </is>
       </c>
     </row>
@@ -4516,7 +4516,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>1.93%</t>
         </is>
       </c>
     </row>
@@ -4543,7 +4543,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.64%</t>
         </is>
       </c>
     </row>
@@ -4570,7 +4570,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -4597,7 +4597,7 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -4624,7 +4624,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -4678,7 +4678,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -4705,7 +4705,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -4732,7 +4732,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4759,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -4786,7 +4786,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -4813,7 +4813,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -4840,7 +4840,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>11.54%</t>
         </is>
       </c>
     </row>
@@ -4867,7 +4867,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>1.92%</t>
         </is>
       </c>
     </row>
@@ -4894,7 +4894,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>1.92%</t>
         </is>
       </c>
     </row>
@@ -4921,7 +4921,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>7.69%</t>
         </is>
       </c>
     </row>
@@ -4948,7 +4948,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>7.69%</t>
         </is>
       </c>
     </row>
@@ -4975,7 +4975,7 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1.28%</t>
         </is>
       </c>
     </row>
@@ -5002,7 +5002,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1.28%</t>
         </is>
       </c>
     </row>
@@ -5029,7 +5029,7 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>1.92%</t>
         </is>
       </c>
     </row>
@@ -5056,7 +5056,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>1.92%</t>
         </is>
       </c>
     </row>
@@ -5083,7 +5083,7 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>7.69%</t>
         </is>
       </c>
     </row>
@@ -5110,7 +5110,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>10.21%</t>
         </is>
       </c>
     </row>
@@ -5137,7 +5137,7 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.08%</t>
         </is>
       </c>
     </row>
@@ -5164,7 +5164,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.08%</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5191,7 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>16.33%</t>
         </is>
       </c>
     </row>
@@ -5218,7 +5218,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>6.12%</t>
         </is>
       </c>
     </row>
@@ -5245,7 +5245,7 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>6.12%</t>
         </is>
       </c>
     </row>
@@ -5272,7 +5272,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.68%</t>
         </is>
       </c>
     </row>
@@ -5299,7 +5299,7 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.68%</t>
         </is>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.04%</t>
         </is>
       </c>
     </row>
@@ -5353,7 +5353,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>4.08%</t>
         </is>
       </c>
     </row>
@@ -5380,7 +5380,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.04%</t>
         </is>
       </c>
     </row>
@@ -5407,7 +5407,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>1%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -5434,7 +5434,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>12.25%</t>
         </is>
       </c>
     </row>
@@ -5461,7 +5461,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>8.17%</t>
         </is>
       </c>
     </row>
@@ -5488,7 +5488,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>8.16%</t>
         </is>
       </c>
     </row>
@@ -5515,7 +5515,7 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1.36%</t>
         </is>
       </c>
     </row>
@@ -5542,7 +5542,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1.36%</t>
         </is>
       </c>
     </row>
@@ -5569,7 +5569,7 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.04%</t>
         </is>
       </c>
     </row>
@@ -5596,7 +5596,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.04%</t>
         </is>
       </c>
     </row>
@@ -5623,7 +5623,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>8.16%</t>
         </is>
       </c>
     </row>
@@ -5650,7 +5650,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>5.59%</t>
         </is>
       </c>
     </row>
@@ -5677,7 +5677,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>13.05%</t>
         </is>
       </c>
     </row>
@@ -5704,7 +5704,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>9.32%</t>
         </is>
       </c>
     </row>
@@ -5731,7 +5731,7 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>9.32%</t>
         </is>
       </c>
     </row>
@@ -5758,7 +5758,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>7.46%</t>
         </is>
       </c>
     </row>
@@ -5785,7 +5785,7 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>9.32%</t>
         </is>
       </c>
     </row>
@@ -5812,7 +5812,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.62%</t>
         </is>
       </c>
     </row>
@@ -5839,7 +5839,7 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.62%</t>
         </is>
       </c>
     </row>
@@ -5866,7 +5866,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.62%</t>
         </is>
       </c>
     </row>
@@ -5893,7 +5893,7 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.62%</t>
         </is>
       </c>
     </row>
@@ -5920,7 +5920,7 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>3.73%</t>
         </is>
       </c>
     </row>
@@ -5947,7 +5947,7 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>11.18%</t>
         </is>
       </c>
     </row>
@@ -5974,7 +5974,7 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>7.45%</t>
         </is>
       </c>
     </row>
@@ -6001,7 +6001,7 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>7.45%</t>
         </is>
       </c>
     </row>
@@ -6028,7 +6028,7 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1.24%</t>
         </is>
       </c>
     </row>
@@ -6055,7 +6055,7 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1.24%</t>
         </is>
       </c>
     </row>
@@ -6082,7 +6082,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>1.86%</t>
         </is>
       </c>
     </row>
@@ -6109,7 +6109,7 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>1.86%</t>
         </is>
       </c>
     </row>
@@ -6136,7 +6136,7 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>7.45%</t>
         </is>
       </c>
     </row>
@@ -6163,7 +6163,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>6.34%</t>
         </is>
       </c>
     </row>
@@ -6190,7 +6190,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>8.45%</t>
         </is>
       </c>
     </row>
@@ -6217,7 +6217,7 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>6.34%</t>
         </is>
       </c>
     </row>
@@ -6244,7 +6244,7 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1.41%</t>
         </is>
       </c>
     </row>
@@ -6271,7 +6271,7 @@
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>30%, 5%</t>
+          <t>4.93%</t>
         </is>
       </c>
     </row>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>2.11%</t>
         </is>
       </c>
     </row>
@@ -6325,7 +6325,7 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>4.23%</t>
         </is>
       </c>
     </row>
@@ -6352,7 +6352,7 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>4.23%</t>
         </is>
       </c>
     </row>
@@ -6379,7 +6379,7 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.11%</t>
         </is>
       </c>
     </row>
@@ -6406,7 +6406,7 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.11%</t>
         </is>
       </c>
     </row>
@@ -6433,7 +6433,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>8.45%</t>
         </is>
       </c>
     </row>
@@ -6460,7 +6460,7 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>12.68%</t>
         </is>
       </c>
     </row>
@@ -6487,7 +6487,7 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.11%</t>
         </is>
       </c>
     </row>
@@ -6514,7 +6514,7 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.11%</t>
         </is>
       </c>
     </row>
@@ -6541,7 +6541,7 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>8.45%</t>
         </is>
       </c>
     </row>
@@ -6568,7 +6568,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>8.45%</t>
         </is>
       </c>
     </row>
@@ -6595,7 +6595,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1.41%</t>
         </is>
       </c>
     </row>
@@ -6622,7 +6622,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1.41%</t>
         </is>
       </c>
     </row>
@@ -6649,7 +6649,7 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.11%</t>
         </is>
       </c>
     </row>
@@ -6676,7 +6676,7 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.11%</t>
         </is>
       </c>
     </row>
@@ -6703,7 +6703,7 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>8.45%</t>
         </is>
       </c>
     </row>
@@ -6730,7 +6730,7 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>5.00%</t>
         </is>
       </c>
     </row>
@@ -6757,7 +6757,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>10.00%</t>
         </is>
       </c>
     </row>
@@ -6784,7 +6784,7 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>5.00%</t>
         </is>
       </c>
     </row>
@@ -6811,7 +6811,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.83%</t>
         </is>
       </c>
     </row>
@@ -6838,7 +6838,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.83%</t>
         </is>
       </c>
     </row>
@@ -6865,7 +6865,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.50%</t>
         </is>
       </c>
     </row>
@@ -6892,7 +6892,7 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.50%</t>
         </is>
       </c>
     </row>
@@ -6919,7 +6919,7 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.50%</t>
         </is>
       </c>
     </row>
@@ -6946,7 +6946,7 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.50%</t>
         </is>
       </c>
     </row>
@@ -6973,7 +6973,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>10.00%</t>
         </is>
       </c>
     </row>
@@ -7000,7 +7000,7 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>15.00%</t>
         </is>
       </c>
     </row>
@@ -7027,7 +7027,7 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.50%</t>
         </is>
       </c>
     </row>
@@ -7054,7 +7054,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.50%</t>
         </is>
       </c>
     </row>
@@ -7081,7 +7081,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>10.00%</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>10.00%</t>
         </is>
       </c>
     </row>
@@ -7135,7 +7135,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1.67%</t>
         </is>
       </c>
     </row>
@@ -7162,7 +7162,7 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1.67%</t>
         </is>
       </c>
     </row>
@@ -7189,7 +7189,7 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.50%</t>
         </is>
       </c>
     </row>
@@ -7216,7 +7216,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.50%</t>
         </is>
       </c>
     </row>
@@ -7243,7 +7243,7 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>10.00%</t>
         </is>
       </c>
     </row>
@@ -7270,7 +7270,7 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -7297,7 +7297,7 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -7324,7 +7324,7 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>28.57%</t>
         </is>
       </c>
     </row>
@@ -7351,7 +7351,7 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>28.57%</t>
         </is>
       </c>
     </row>
@@ -7378,7 +7378,7 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>28.57%</t>
         </is>
       </c>
     </row>
@@ -7405,7 +7405,7 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>14.29%</t>
         </is>
       </c>
     </row>
@@ -7432,7 +7432,7 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -7459,7 +7459,7 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -7486,7 +7486,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>16.67%</t>
         </is>
       </c>
     </row>
@@ -7513,7 +7513,7 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>16.67%</t>
         </is>
       </c>
     </row>
@@ -7540,7 +7540,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -7567,7 +7567,7 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -7594,7 +7594,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -7621,7 +7621,7 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -7648,7 +7648,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>57.14%</t>
         </is>
       </c>
     </row>
@@ -7675,7 +7675,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>28.57%</t>
         </is>
       </c>
     </row>
@@ -7702,7 +7702,7 @@
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>14.29%</t>
         </is>
       </c>
     </row>
@@ -7729,7 +7729,7 @@
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>28.57%</t>
         </is>
       </c>
     </row>
@@ -7756,7 +7756,7 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>28.57%</t>
         </is>
       </c>
     </row>
@@ -7783,7 +7783,7 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>28.57%</t>
         </is>
       </c>
     </row>
@@ -7810,7 +7810,7 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>14.29%</t>
         </is>
       </c>
     </row>
@@ -7837,7 +7837,7 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -7864,7 +7864,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -7891,7 +7891,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>16.67%</t>
         </is>
       </c>
     </row>
@@ -7918,7 +7918,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>16.67%</t>
         </is>
       </c>
     </row>
@@ -7945,7 +7945,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -7972,7 +7972,7 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -7999,7 +7999,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>27.91%</t>
         </is>
       </c>
     </row>
@@ -8026,7 +8026,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>9.30%</t>
         </is>
       </c>
     </row>
@@ -8053,7 +8053,7 @@
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.65%</t>
         </is>
       </c>
     </row>
@@ -8080,7 +8080,7 @@
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>9.30%</t>
         </is>
       </c>
     </row>
@@ -8107,7 +8107,7 @@
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>6.98%</t>
         </is>
       </c>
     </row>
@@ -8134,7 +8134,7 @@
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>6.98%</t>
         </is>
       </c>
     </row>
@@ -8161,7 +8161,7 @@
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.78%</t>
         </is>
       </c>
     </row>
@@ -8188,7 +8188,7 @@
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.77%</t>
         </is>
       </c>
     </row>
@@ -8215,7 +8215,7 @@
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.77%</t>
         </is>
       </c>
     </row>
@@ -8242,7 +8242,7 @@
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.33%</t>
         </is>
       </c>
     </row>
@@ -8269,7 +8269,7 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>4.65%</t>
         </is>
       </c>
     </row>
@@ -8296,7 +8296,7 @@
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.33%</t>
         </is>
       </c>
     </row>
@@ -8323,7 +8323,7 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -8350,7 +8350,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -8377,7 +8377,7 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -8404,7 +8404,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -8431,7 +8431,7 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -8458,7 +8458,7 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -8485,7 +8485,7 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -8512,7 +8512,7 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -8539,7 +8539,7 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -8566,7 +8566,7 @@
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>13.95%</t>
         </is>
       </c>
     </row>
@@ -8593,7 +8593,7 @@
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>9.30%</t>
         </is>
       </c>
     </row>
@@ -8620,7 +8620,7 @@
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>11.81%</t>
         </is>
       </c>
     </row>
@@ -8647,7 +8647,7 @@
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.73%</t>
         </is>
       </c>
     </row>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.73%</t>
         </is>
       </c>
     </row>
@@ -8701,7 +8701,7 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>30%, 5%</t>
+          <t>5.51%</t>
         </is>
       </c>
     </row>
@@ -8728,7 +8728,7 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>15%, 30%, 5%</t>
+          <t>10.24%</t>
         </is>
       </c>
     </row>
@@ -8755,7 +8755,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.72%</t>
         </is>
       </c>
     </row>
@@ -8782,7 +8782,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>7.09%</t>
         </is>
       </c>
     </row>
@@ -8809,7 +8809,7 @@
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>15%, 5%</t>
+          <t>3.15%</t>
         </is>
       </c>
     </row>
@@ -8836,7 +8836,7 @@
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.79%</t>
         </is>
       </c>
     </row>
@@ -8863,7 +8863,7 @@
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.36%</t>
         </is>
       </c>
     </row>
@@ -8890,7 +8890,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>2.36%</t>
         </is>
       </c>
     </row>
@@ -8917,7 +8917,7 @@
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -8944,7 +8944,7 @@
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>9.45%</t>
         </is>
       </c>
     </row>
@@ -8971,7 +8971,7 @@
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>9.45%</t>
         </is>
       </c>
     </row>
@@ -8998,7 +8998,7 @@
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>9.45%</t>
         </is>
       </c>
     </row>
@@ -9025,7 +9025,7 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>4.72%</t>
         </is>
       </c>
     </row>
@@ -9052,7 +9052,7 @@
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.72%</t>
         </is>
       </c>
     </row>
@@ -9079,7 +9079,7 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>4.72%</t>
         </is>
       </c>
     </row>
@@ -9106,7 +9106,7 @@
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>10.00%</t>
         </is>
       </c>
     </row>
@@ -9133,7 +9133,7 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>6.67%</t>
         </is>
       </c>
     </row>
@@ -9160,7 +9160,7 @@
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>6.67%</t>
         </is>
       </c>
     </row>
@@ -9187,7 +9187,7 @@
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>10.00%</t>
         </is>
       </c>
     </row>
@@ -9214,7 +9214,7 @@
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>3.33%</t>
         </is>
       </c>
     </row>
@@ -9241,7 +9241,7 @@
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>3.33%</t>
         </is>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -9295,7 +9295,7 @@
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -9322,7 +9322,7 @@
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -9349,7 +9349,7 @@
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>16.67%</t>
         </is>
       </c>
     </row>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -9403,7 +9403,7 @@
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -9430,7 +9430,7 @@
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -9457,7 +9457,7 @@
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -9484,7 +9484,7 @@
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -9511,7 +9511,7 @@
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -9538,7 +9538,7 @@
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -9565,7 +9565,7 @@
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>26.67%</t>
         </is>
       </c>
     </row>
@@ -9592,7 +9592,7 @@
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>20.00%</t>
         </is>
       </c>
     </row>
@@ -9619,7 +9619,7 @@
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>13.33%</t>
         </is>
       </c>
     </row>
@@ -9646,7 +9646,7 @@
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>9.68%</t>
         </is>
       </c>
     </row>
@@ -9673,7 +9673,7 @@
       </c>
       <c r="E343" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>29.03%</t>
         </is>
       </c>
     </row>
@@ -9700,7 +9700,7 @@
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1.61%</t>
         </is>
       </c>
     </row>
@@ -9727,7 +9727,7 @@
       </c>
       <c r="E345" t="inlineStr">
         <is>
-          <t>15%, 5%</t>
+          <t>6.45%</t>
         </is>
       </c>
     </row>
@@ -9754,7 +9754,7 @@
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>4.84%</t>
         </is>
       </c>
     </row>
@@ -9781,7 +9781,7 @@
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>4.84%</t>
         </is>
       </c>
     </row>
@@ -9808,7 +9808,7 @@
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>4.84%</t>
         </is>
       </c>
     </row>
@@ -9835,7 +9835,7 @@
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -9862,7 +9862,7 @@
       </c>
       <c r="E350" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>40.00%</t>
         </is>
       </c>
     </row>
@@ -9889,7 +9889,7 @@
       </c>
       <c r="E351" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>40.00%</t>
         </is>
       </c>
     </row>
@@ -9916,7 +9916,7 @@
       </c>
       <c r="E352" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>20.00%</t>
         </is>
       </c>
     </row>
@@ -9943,7 +9943,7 @@
       </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -9970,7 +9970,7 @@
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -9997,7 +9997,7 @@
       </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -10024,7 +10024,7 @@
       </c>
       <c r="E356" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>19.35%</t>
         </is>
       </c>
     </row>
@@ -10051,7 +10051,7 @@
       </c>
       <c r="E357" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>9.68%</t>
         </is>
       </c>
     </row>
@@ -10078,7 +10078,7 @@
       </c>
       <c r="E358" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>9.68%</t>
         </is>
       </c>
     </row>
@@ -10105,7 +10105,7 @@
       </c>
       <c r="E359" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>19.05%</t>
         </is>
       </c>
     </row>
@@ -10132,7 +10132,7 @@
       </c>
       <c r="E360" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>38.10%</t>
         </is>
       </c>
     </row>
@@ -10159,7 +10159,7 @@
       </c>
       <c r="E361" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>19.05%</t>
         </is>
       </c>
     </row>
@@ -10186,7 +10186,7 @@
       </c>
       <c r="E362" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>3.17%</t>
         </is>
       </c>
     </row>
@@ -10213,7 +10213,7 @@
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1.59%</t>
         </is>
       </c>
     </row>
@@ -10240,7 +10240,7 @@
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>9.52%</t>
         </is>
       </c>
     </row>
@@ -10267,7 +10267,7 @@
       </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>9.52%</t>
         </is>
       </c>
     </row>
@@ -10294,7 +10294,7 @@
       </c>
       <c r="E366" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>15.19%</t>
         </is>
       </c>
     </row>
@@ -10321,7 +10321,7 @@
       </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>15.19%</t>
         </is>
       </c>
     </row>
@@ -10348,7 +10348,7 @@
       </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>3.80%</t>
         </is>
       </c>
     </row>
@@ -10375,7 +10375,7 @@
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>15.19%</t>
         </is>
       </c>
     </row>
@@ -10402,7 +10402,7 @@
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>15.19%</t>
         </is>
       </c>
     </row>
@@ -10429,7 +10429,7 @@
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>2.53%</t>
         </is>
       </c>
     </row>
@@ -10456,7 +10456,7 @@
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>2.53%</t>
         </is>
       </c>
     </row>
@@ -10483,7 +10483,7 @@
       </c>
       <c r="E373" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>3.80%</t>
         </is>
       </c>
     </row>
@@ -10510,7 +10510,7 @@
       </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>3.80%</t>
         </is>
       </c>
     </row>
@@ -10537,7 +10537,7 @@
       </c>
       <c r="E375" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>7.60%</t>
         </is>
       </c>
     </row>
@@ -10564,7 +10564,7 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>7.59%</t>
         </is>
       </c>
     </row>
@@ -10591,7 +10591,7 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>7.59%</t>
         </is>
       </c>
     </row>
@@ -10618,7 +10618,7 @@
       </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -10645,7 +10645,7 @@
       </c>
       <c r="E379" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -10672,7 +10672,7 @@
       </c>
       <c r="E380" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -10699,7 +10699,7 @@
       </c>
       <c r="E381" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -10726,7 +10726,7 @@
       </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -10753,7 +10753,7 @@
       </c>
       <c r="E383" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -10780,7 +10780,7 @@
       </c>
       <c r="E384" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -10807,7 +10807,7 @@
       </c>
       <c r="E385" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -10834,7 +10834,7 @@
       </c>
       <c r="E386" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -10861,7 +10861,7 @@
       </c>
       <c r="E387" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -10888,7 +10888,7 @@
       </c>
       <c r="E388" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -10915,7 +10915,7 @@
       </c>
       <c r="E389" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -10942,7 +10942,7 @@
       </c>
       <c r="E390" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>28.57%</t>
         </is>
       </c>
     </row>
@@ -10969,7 +10969,7 @@
       </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>28.57%</t>
         </is>
       </c>
     </row>
@@ -10996,7 +10996,7 @@
       </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>28.57%</t>
         </is>
       </c>
     </row>
@@ -11023,7 +11023,7 @@
       </c>
       <c r="E393" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>14.29%</t>
         </is>
       </c>
     </row>
@@ -11050,7 +11050,7 @@
       </c>
       <c r="E394" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -11077,7 +11077,7 @@
       </c>
       <c r="E395" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -11104,7 +11104,7 @@
       </c>
       <c r="E396" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>16.67%</t>
         </is>
       </c>
     </row>
@@ -11131,7 +11131,7 @@
       </c>
       <c r="E397" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>16.67%</t>
         </is>
       </c>
     </row>
@@ -11158,7 +11158,7 @@
       </c>
       <c r="E398" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -11185,7 +11185,7 @@
       </c>
       <c r="E399" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -11212,7 +11212,7 @@
       </c>
       <c r="E400" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -11239,7 +11239,7 @@
       </c>
       <c r="E401" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -11266,7 +11266,7 @@
       </c>
       <c r="E402" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>28.57%</t>
         </is>
       </c>
     </row>
@@ -11293,7 +11293,7 @@
       </c>
       <c r="E403" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>28.57%</t>
         </is>
       </c>
     </row>
@@ -11320,7 +11320,7 @@
       </c>
       <c r="E404" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>28.57%</t>
         </is>
       </c>
     </row>
@@ -11347,7 +11347,7 @@
       </c>
       <c r="E405" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>14.29%</t>
         </is>
       </c>
     </row>
@@ -11374,7 +11374,7 @@
       </c>
       <c r="E406" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -11401,7 +11401,7 @@
       </c>
       <c r="E407" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -11428,7 +11428,7 @@
       </c>
       <c r="E408" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>16.67%</t>
         </is>
       </c>
     </row>
@@ -11455,7 +11455,7 @@
       </c>
       <c r="E409" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>16.67%</t>
         </is>
       </c>
     </row>
@@ -11482,7 +11482,7 @@
       </c>
       <c r="E410" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -11509,7 +11509,7 @@
       </c>
       <c r="E411" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -11536,7 +11536,7 @@
       </c>
       <c r="E412" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -11563,7 +11563,7 @@
       </c>
       <c r="E413" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -11590,7 +11590,7 @@
       </c>
       <c r="E414" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -11617,7 +11617,7 @@
       </c>
       <c r="E415" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -11644,7 +11644,7 @@
       </c>
       <c r="E416" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -11671,7 +11671,7 @@
       </c>
       <c r="E417" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>40.00%</t>
         </is>
       </c>
     </row>
@@ -11698,7 +11698,7 @@
       </c>
       <c r="E418" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>40.00%</t>
         </is>
       </c>
     </row>
@@ -11725,7 +11725,7 @@
       </c>
       <c r="E419" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>20.00%</t>
         </is>
       </c>
     </row>
@@ -11752,7 +11752,7 @@
       </c>
       <c r="E420" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -11779,7 +11779,7 @@
       </c>
       <c r="E421" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -11806,7 +11806,7 @@
       </c>
       <c r="E422" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -11833,7 +11833,7 @@
       </c>
       <c r="E423" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -11860,7 +11860,7 @@
       </c>
       <c r="E424" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -11887,7 +11887,7 @@
       </c>
       <c r="E425" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -11914,7 +11914,7 @@
       </c>
       <c r="E426" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -11941,7 +11941,7 @@
       </c>
       <c r="E427" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -11968,7 +11968,7 @@
       </c>
       <c r="E428" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -11995,7 +11995,7 @@
       </c>
       <c r="E429" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -12022,7 +12022,7 @@
       </c>
       <c r="E430" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -12049,7 +12049,7 @@
       </c>
       <c r="E431" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -12076,7 +12076,7 @@
       </c>
       <c r="E432" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -12103,7 +12103,7 @@
       </c>
       <c r="E433" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>16.36%</t>
         </is>
       </c>
     </row>
@@ -12130,7 +12130,7 @@
       </c>
       <c r="E434" t="inlineStr">
         <is>
-          <t>15%, 30%, 5%</t>
+          <t>11.52%</t>
         </is>
       </c>
     </row>
@@ -12157,7 +12157,7 @@
       </c>
       <c r="E435" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>16.36%</t>
         </is>
       </c>
     </row>
@@ -12184,7 +12184,7 @@
       </c>
       <c r="E436" t="inlineStr">
         <is>
-          <t>15%, 30%, 5%</t>
+          <t>11.51%</t>
         </is>
       </c>
     </row>
@@ -12211,7 +12211,7 @@
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t>30%, 5%</t>
+          <t>4.24%</t>
         </is>
       </c>
     </row>
@@ -12238,7 +12238,7 @@
       </c>
       <c r="E438" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>7.27%</t>
         </is>
       </c>
     </row>
@@ -12265,7 +12265,7 @@
       </c>
       <c r="E439" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>3.64%</t>
         </is>
       </c>
     </row>
@@ -12292,7 +12292,7 @@
       </c>
       <c r="E440" t="inlineStr">
         <is>
-          <t>15%, 5%</t>
+          <t>2.42%</t>
         </is>
       </c>
     </row>
@@ -12319,7 +12319,7 @@
       </c>
       <c r="E441" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>0.61%</t>
         </is>
       </c>
     </row>
@@ -12346,7 +12346,7 @@
       </c>
       <c r="E442" t="inlineStr">
         <is>
-          <t>30%, 5%</t>
+          <t>7.88%</t>
         </is>
       </c>
     </row>
@@ -12373,7 +12373,7 @@
       </c>
       <c r="E443" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>1.82%</t>
         </is>
       </c>
     </row>
@@ -12400,7 +12400,7 @@
       </c>
       <c r="E444" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -12427,7 +12427,7 @@
       </c>
       <c r="E445" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -12454,7 +12454,7 @@
       </c>
       <c r="E446" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -12481,7 +12481,7 @@
       </c>
       <c r="E447" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -12508,7 +12508,7 @@
       </c>
       <c r="E448" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -12535,7 +12535,7 @@
       </c>
       <c r="E449" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -12562,7 +12562,7 @@
       </c>
       <c r="E450" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -12589,7 +12589,7 @@
       </c>
       <c r="E451" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -12616,7 +12616,7 @@
       </c>
       <c r="E452" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -12643,7 +12643,7 @@
       </c>
       <c r="E453" t="inlineStr">
         <is>
-          <t>1%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -12670,7 +12670,7 @@
       </c>
       <c r="E454" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>7.27%</t>
         </is>
       </c>
     </row>
@@ -12697,7 +12697,7 @@
       </c>
       <c r="E455" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>1.82%</t>
         </is>
       </c>
     </row>
@@ -12724,7 +12724,7 @@
       </c>
       <c r="E456" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1.82%</t>
         </is>
       </c>
     </row>
@@ -12751,7 +12751,7 @@
       </c>
       <c r="E457" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>1.82%</t>
         </is>
       </c>
     </row>
@@ -12778,7 +12778,7 @@
       </c>
       <c r="E458" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>3.64%</t>
         </is>
       </c>
     </row>
@@ -12805,7 +12805,7 @@
       </c>
       <c r="E459" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -12832,7 +12832,7 @@
       </c>
       <c r="E460" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -12859,7 +12859,7 @@
       </c>
       <c r="E461" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -12886,7 +12886,7 @@
       </c>
       <c r="E462" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -12913,7 +12913,7 @@
       </c>
       <c r="E463" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -12940,7 +12940,7 @@
       </c>
       <c r="E464" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -12967,7 +12967,7 @@
       </c>
       <c r="E465" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -12994,7 +12994,7 @@
       </c>
       <c r="E466" t="inlineStr">
         <is>
-          <t>1%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -13021,7 +13021,7 @@
       </c>
       <c r="E467" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>15.19%</t>
         </is>
       </c>
     </row>
@@ -13048,7 +13048,7 @@
       </c>
       <c r="E468" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>22.78%</t>
         </is>
       </c>
     </row>
@@ -13075,7 +13075,7 @@
       </c>
       <c r="E469" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>3.80%</t>
         </is>
       </c>
     </row>
@@ -13102,7 +13102,7 @@
       </c>
       <c r="E470" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>15.19%</t>
         </is>
       </c>
     </row>
@@ -13129,7 +13129,7 @@
       </c>
       <c r="E471" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>15.19%</t>
         </is>
       </c>
     </row>
@@ -13156,7 +13156,7 @@
       </c>
       <c r="E472" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>2.53%</t>
         </is>
       </c>
     </row>
@@ -13183,7 +13183,7 @@
       </c>
       <c r="E473" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>2.53%</t>
         </is>
       </c>
     </row>
@@ -13210,7 +13210,7 @@
       </c>
       <c r="E474" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>3.80%</t>
         </is>
       </c>
     </row>
@@ -13237,7 +13237,7 @@
       </c>
       <c r="E475" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>3.80%</t>
         </is>
       </c>
     </row>
@@ -13264,7 +13264,7 @@
       </c>
       <c r="E476" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>15.19%</t>
         </is>
       </c>
     </row>
@@ -13291,7 +13291,7 @@
       </c>
       <c r="E477" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -13318,7 +13318,7 @@
       </c>
       <c r="E478" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -13345,7 +13345,7 @@
       </c>
       <c r="E479" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -13372,7 +13372,7 @@
       </c>
       <c r="E480" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -13399,7 +13399,7 @@
       </c>
       <c r="E481" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>16.67%</t>
         </is>
       </c>
     </row>
@@ -13426,7 +13426,7 @@
       </c>
       <c r="E482" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>16.67%</t>
         </is>
       </c>
     </row>
@@ -13453,7 +13453,7 @@
       </c>
       <c r="E483" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -13480,7 +13480,7 @@
       </c>
       <c r="E484" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -13507,7 +13507,7 @@
       </c>
       <c r="E485" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>16.67%</t>
         </is>
       </c>
     </row>
@@ -13534,7 +13534,7 @@
       </c>
       <c r="E486" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>16.67%</t>
         </is>
       </c>
     </row>
@@ -13561,7 +13561,7 @@
       </c>
       <c r="E487" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -13588,7 +13588,7 @@
       </c>
       <c r="E488" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -13615,7 +13615,7 @@
       </c>
       <c r="E489" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>33.34%</t>
         </is>
       </c>
     </row>
@@ -13642,7 +13642,7 @@
       </c>
       <c r="E490" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -13669,7 +13669,7 @@
       </c>
       <c r="E491" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -13696,7 +13696,7 @@
       </c>
       <c r="E492" t="inlineStr">
         <is>
-          <t>1%</t>
+          <t>33.34%</t>
         </is>
       </c>
     </row>
@@ -13723,7 +13723,7 @@
       </c>
       <c r="E493" t="inlineStr">
         <is>
-          <t>1%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -13750,7 +13750,7 @@
       </c>
       <c r="E494" t="inlineStr">
         <is>
-          <t>1%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -13777,7 +13777,7 @@
       </c>
       <c r="E495" t="inlineStr">
         <is>
-          <t>15%, 30%</t>
+          <t>60.00%</t>
         </is>
       </c>
     </row>
@@ -13804,7 +13804,7 @@
       </c>
       <c r="E496" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>40.00%</t>
         </is>
       </c>
     </row>
@@ -13831,7 +13831,7 @@
       </c>
       <c r="E497" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -13858,7 +13858,7 @@
       </c>
       <c r="E498" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -13885,7 +13885,7 @@
       </c>
       <c r="E499" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -13912,7 +13912,7 @@
       </c>
       <c r="E500" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -13939,7 +13939,7 @@
       </c>
       <c r="E501" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>25.00%</t>
         </is>
       </c>
     </row>
@@ -13966,7 +13966,7 @@
       </c>
       <c r="E502" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -13993,7 +13993,7 @@
       </c>
       <c r="E503" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>50.00%</t>
         </is>
       </c>
     </row>
@@ -14020,7 +14020,7 @@
       </c>
       <c r="E504" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>66.67%</t>
         </is>
       </c>
     </row>
@@ -14047,7 +14047,7 @@
       </c>
       <c r="E505" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -14074,7 +14074,7 @@
       </c>
       <c r="E506" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>
@@ -14101,7 +14101,7 @@
       </c>
       <c r="E507" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>100.00%</t>
         </is>
       </c>
     </row>

</xml_diff>